<commit_message>
chore: 🗃️ Regenera matriz de nós e planilha de cobertura
node_matrix.txt estava desatualizado: os drivers condicionais
(BENCH_DURACAO) adicionados aos benchmarks inseriram While/Break/
AugAssign/Add em quase todos os fontes e a matriz não foi regerada.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/arquivos/xlsx/nos_ast_cobertos.xlsx
+++ b/arquivos/xlsx/nos_ast_cobertos.xlsx
@@ -1011,12 +1011,12 @@
       <c r="F2" s="3" t="n"/>
       <c r="G2" s="4" t="n"/>
       <c r="H2" s="3" t="n"/>
-      <c r="I2" s="4" t="n"/>
+      <c r="I2" s="3" t="n"/>
       <c r="J2" s="4" t="n"/>
       <c r="K2" s="4" t="n"/>
-      <c r="L2" s="4" t="n"/>
+      <c r="L2" s="3" t="n"/>
       <c r="M2" s="4" t="n"/>
-      <c r="N2" s="4" t="n"/>
+      <c r="N2" s="3" t="n"/>
       <c r="O2" s="3" t="n"/>
       <c r="P2" s="4" t="n"/>
       <c r="Q2" s="4" t="n"/>
@@ -1031,7 +1031,7 @@
       <c r="Z2" s="4" t="n"/>
       <c r="AA2" s="3" t="n"/>
       <c r="AB2" s="4" t="n"/>
-      <c r="AC2" s="4" t="n"/>
+      <c r="AC2" s="3" t="n"/>
       <c r="AD2" s="4" t="n"/>
       <c r="AE2" s="4" t="n"/>
       <c r="AF2" s="4" t="n"/>
@@ -1054,16 +1054,16 @@
       <c r="AW2" s="3" t="n"/>
       <c r="AX2" s="3" t="n"/>
       <c r="AY2" s="3" t="n"/>
-      <c r="AZ2" s="4" t="n"/>
+      <c r="AZ2" s="3" t="n"/>
       <c r="BA2" s="4" t="n"/>
       <c r="BB2" s="3" t="n"/>
-      <c r="BC2" s="4" t="n"/>
-      <c r="BD2" s="4" t="n"/>
+      <c r="BC2" s="3" t="n"/>
+      <c r="BD2" s="3" t="n"/>
       <c r="BE2" s="4" t="n"/>
       <c r="BF2" s="3" t="n"/>
       <c r="BG2" s="3" t="n"/>
       <c r="BH2" s="4" t="n"/>
-      <c r="BI2" s="4" t="n"/>
+      <c r="BI2" s="3" t="n"/>
       <c r="BJ2" s="3" t="n"/>
       <c r="BK2" s="3" t="n"/>
       <c r="BL2" s="3" t="n"/>
@@ -1084,11 +1084,11 @@
       <c r="CA2" s="4" t="n"/>
       <c r="CB2" s="3" t="n"/>
       <c r="CC2" s="4" t="n"/>
-      <c r="CD2" s="4" t="n"/>
+      <c r="CD2" s="3" t="n"/>
       <c r="CE2" s="4" t="n"/>
       <c r="CF2" s="4" t="n"/>
-      <c r="CG2" s="4" t="n"/>
-      <c r="CH2" s="4" t="n"/>
+      <c r="CG2" s="3" t="n"/>
+      <c r="CH2" s="3" t="n"/>
       <c r="CI2" s="4" t="n"/>
       <c r="CJ2" s="4" t="n"/>
       <c r="CK2" s="4" t="n"/>
@@ -1125,12 +1125,12 @@
       <c r="F3" s="5" t="n"/>
       <c r="G3" s="4" t="n"/>
       <c r="H3" s="5" t="n"/>
-      <c r="I3" s="4" t="n"/>
+      <c r="I3" s="5" t="n"/>
       <c r="J3" s="4" t="n"/>
       <c r="K3" s="4" t="n"/>
-      <c r="L3" s="4" t="n"/>
+      <c r="L3" s="5" t="n"/>
       <c r="M3" s="4" t="n"/>
-      <c r="N3" s="4" t="n"/>
+      <c r="N3" s="5" t="n"/>
       <c r="O3" s="5" t="n"/>
       <c r="P3" s="4" t="n"/>
       <c r="Q3" s="4" t="n"/>
@@ -1145,7 +1145,7 @@
       <c r="Z3" s="4" t="n"/>
       <c r="AA3" s="5" t="n"/>
       <c r="AB3" s="4" t="n"/>
-      <c r="AC3" s="4" t="n"/>
+      <c r="AC3" s="5" t="n"/>
       <c r="AD3" s="4" t="n"/>
       <c r="AE3" s="4" t="n"/>
       <c r="AF3" s="4" t="n"/>
@@ -1168,16 +1168,16 @@
       <c r="AW3" s="5" t="n"/>
       <c r="AX3" s="5" t="n"/>
       <c r="AY3" s="5" t="n"/>
-      <c r="AZ3" s="4" t="n"/>
+      <c r="AZ3" s="5" t="n"/>
       <c r="BA3" s="4" t="n"/>
       <c r="BB3" s="5" t="n"/>
-      <c r="BC3" s="4" t="n"/>
-      <c r="BD3" s="4" t="n"/>
+      <c r="BC3" s="5" t="n"/>
+      <c r="BD3" s="5" t="n"/>
       <c r="BE3" s="4" t="n"/>
       <c r="BF3" s="5" t="n"/>
       <c r="BG3" s="5" t="n"/>
       <c r="BH3" s="4" t="n"/>
-      <c r="BI3" s="3" t="n"/>
+      <c r="BI3" s="5" t="n"/>
       <c r="BJ3" s="5" t="n"/>
       <c r="BK3" s="5" t="n"/>
       <c r="BL3" s="5" t="n"/>
@@ -1198,11 +1198,11 @@
       <c r="CA3" s="4" t="n"/>
       <c r="CB3" s="5" t="n"/>
       <c r="CC3" s="4" t="n"/>
-      <c r="CD3" s="4" t="n"/>
+      <c r="CD3" s="5" t="n"/>
       <c r="CE3" s="4" t="n"/>
       <c r="CF3" s="4" t="n"/>
-      <c r="CG3" s="4" t="n"/>
-      <c r="CH3" s="4" t="n"/>
+      <c r="CG3" s="5" t="n"/>
+      <c r="CH3" s="5" t="n"/>
       <c r="CI3" s="4" t="n"/>
       <c r="CJ3" s="4" t="n"/>
       <c r="CK3" s="4" t="n"/>
@@ -1239,12 +1239,12 @@
       <c r="F4" s="5" t="n"/>
       <c r="G4" s="4" t="n"/>
       <c r="H4" s="5" t="n"/>
-      <c r="I4" s="4" t="n"/>
+      <c r="I4" s="5" t="n"/>
       <c r="J4" s="4" t="n"/>
       <c r="K4" s="4" t="n"/>
-      <c r="L4" s="4" t="n"/>
+      <c r="L4" s="5" t="n"/>
       <c r="M4" s="4" t="n"/>
-      <c r="N4" s="4" t="n"/>
+      <c r="N4" s="5" t="n"/>
       <c r="O4" s="5" t="n"/>
       <c r="P4" s="4" t="n"/>
       <c r="Q4" s="4" t="n"/>
@@ -1259,7 +1259,7 @@
       <c r="Z4" s="4" t="n"/>
       <c r="AA4" s="5" t="n"/>
       <c r="AB4" s="4" t="n"/>
-      <c r="AC4" s="4" t="n"/>
+      <c r="AC4" s="5" t="n"/>
       <c r="AD4" s="4" t="n"/>
       <c r="AE4" s="4" t="n"/>
       <c r="AF4" s="4" t="n"/>
@@ -1282,11 +1282,11 @@
       <c r="AW4" s="5" t="n"/>
       <c r="AX4" s="5" t="n"/>
       <c r="AY4" s="5" t="n"/>
-      <c r="AZ4" s="3" t="n"/>
+      <c r="AZ4" s="5" t="n"/>
       <c r="BA4" s="4" t="n"/>
       <c r="BB4" s="5" t="n"/>
-      <c r="BC4" s="4" t="n"/>
-      <c r="BD4" s="4" t="n"/>
+      <c r="BC4" s="5" t="n"/>
+      <c r="BD4" s="5" t="n"/>
       <c r="BE4" s="4" t="n"/>
       <c r="BF4" s="5" t="n"/>
       <c r="BG4" s="5" t="n"/>
@@ -1312,11 +1312,11 @@
       <c r="CA4" s="4" t="n"/>
       <c r="CB4" s="5" t="n"/>
       <c r="CC4" s="4" t="n"/>
-      <c r="CD4" s="4" t="n"/>
+      <c r="CD4" s="5" t="n"/>
       <c r="CE4" s="4" t="n"/>
       <c r="CF4" s="4" t="n"/>
-      <c r="CG4" s="4" t="n"/>
-      <c r="CH4" s="4" t="n"/>
+      <c r="CG4" s="5" t="n"/>
+      <c r="CH4" s="5" t="n"/>
       <c r="CI4" s="4" t="n"/>
       <c r="CJ4" s="4" t="n"/>
       <c r="CK4" s="4" t="n"/>
@@ -1353,12 +1353,12 @@
       <c r="F5" s="5" t="n"/>
       <c r="G5" s="4" t="n"/>
       <c r="H5" s="5" t="n"/>
-      <c r="I5" s="4" t="n"/>
+      <c r="I5" s="5" t="n"/>
       <c r="J5" s="4" t="n"/>
       <c r="K5" s="4" t="n"/>
-      <c r="L5" s="4" t="n"/>
+      <c r="L5" s="5" t="n"/>
       <c r="M5" s="4" t="n"/>
-      <c r="N5" s="4" t="n"/>
+      <c r="N5" s="5" t="n"/>
       <c r="O5" s="5" t="n"/>
       <c r="P5" s="4" t="n"/>
       <c r="Q5" s="4" t="n"/>
@@ -1373,7 +1373,7 @@
       <c r="Z5" s="4" t="n"/>
       <c r="AA5" s="5" t="n"/>
       <c r="AB5" s="4" t="n"/>
-      <c r="AC5" s="4" t="n"/>
+      <c r="AC5" s="5" t="n"/>
       <c r="AD5" s="4" t="n"/>
       <c r="AE5" s="4" t="n"/>
       <c r="AF5" s="4" t="n"/>
@@ -1399,8 +1399,8 @@
       <c r="AZ5" s="5" t="n"/>
       <c r="BA5" s="4" t="n"/>
       <c r="BB5" s="5" t="n"/>
-      <c r="BC5" s="4" t="n"/>
-      <c r="BD5" s="3" t="n"/>
+      <c r="BC5" s="5" t="n"/>
+      <c r="BD5" s="5" t="n"/>
       <c r="BE5" s="4" t="n"/>
       <c r="BF5" s="5" t="n"/>
       <c r="BG5" s="5" t="n"/>
@@ -1426,11 +1426,11 @@
       <c r="CA5" s="4" t="n"/>
       <c r="CB5" s="5" t="n"/>
       <c r="CC5" s="4" t="n"/>
-      <c r="CD5" s="4" t="n"/>
+      <c r="CD5" s="5" t="n"/>
       <c r="CE5" s="4" t="n"/>
       <c r="CF5" s="4" t="n"/>
-      <c r="CG5" s="4" t="n"/>
-      <c r="CH5" s="4" t="n"/>
+      <c r="CG5" s="5" t="n"/>
+      <c r="CH5" s="5" t="n"/>
       <c r="CI5" s="4" t="n"/>
       <c r="CJ5" s="4" t="n"/>
       <c r="CK5" s="4" t="n"/>
@@ -1467,12 +1467,12 @@
       <c r="F6" s="5" t="n"/>
       <c r="G6" s="4" t="n"/>
       <c r="H6" s="5" t="n"/>
-      <c r="I6" s="4" t="n"/>
+      <c r="I6" s="5" t="n"/>
       <c r="J6" s="4" t="n"/>
       <c r="K6" s="4" t="n"/>
-      <c r="L6" s="4" t="n"/>
+      <c r="L6" s="5" t="n"/>
       <c r="M6" s="4" t="n"/>
-      <c r="N6" s="4" t="n"/>
+      <c r="N6" s="5" t="n"/>
       <c r="O6" s="5" t="n"/>
       <c r="P6" s="4" t="n"/>
       <c r="Q6" s="4" t="n"/>
@@ -1487,7 +1487,7 @@
       <c r="Z6" s="4" t="n"/>
       <c r="AA6" s="5" t="n"/>
       <c r="AB6" s="4" t="n"/>
-      <c r="AC6" s="4" t="n"/>
+      <c r="AC6" s="5" t="n"/>
       <c r="AD6" s="4" t="n"/>
       <c r="AE6" s="3" t="n"/>
       <c r="AF6" s="4" t="n"/>
@@ -1513,7 +1513,7 @@
       <c r="AZ6" s="5" t="n"/>
       <c r="BA6" s="4" t="n"/>
       <c r="BB6" s="5" t="n"/>
-      <c r="BC6" s="4" t="n"/>
+      <c r="BC6" s="5" t="n"/>
       <c r="BD6" s="5" t="n"/>
       <c r="BE6" s="4" t="n"/>
       <c r="BF6" s="5" t="n"/>
@@ -1540,11 +1540,11 @@
       <c r="CA6" s="3" t="n"/>
       <c r="CB6" s="5" t="n"/>
       <c r="CC6" s="4" t="n"/>
-      <c r="CD6" s="4" t="n"/>
+      <c r="CD6" s="5" t="n"/>
       <c r="CE6" s="4" t="n"/>
       <c r="CF6" s="3" t="n"/>
-      <c r="CG6" s="3" t="n"/>
-      <c r="CH6" s="4" t="n"/>
+      <c r="CG6" s="5" t="n"/>
+      <c r="CH6" s="5" t="n"/>
       <c r="CI6" s="4" t="n"/>
       <c r="CJ6" s="4" t="n"/>
       <c r="CK6" s="4" t="n"/>
@@ -1581,12 +1581,12 @@
       <c r="F7" s="5" t="n"/>
       <c r="G7" s="4" t="n"/>
       <c r="H7" s="5" t="n"/>
-      <c r="I7" s="4" t="n"/>
+      <c r="I7" s="5" t="n"/>
       <c r="J7" s="4" t="n"/>
       <c r="K7" s="4" t="n"/>
-      <c r="L7" s="4" t="n"/>
+      <c r="L7" s="5" t="n"/>
       <c r="M7" s="4" t="n"/>
-      <c r="N7" s="4" t="n"/>
+      <c r="N7" s="5" t="n"/>
       <c r="O7" s="5" t="n"/>
       <c r="P7" s="4" t="n"/>
       <c r="Q7" s="4" t="n"/>
@@ -1601,7 +1601,7 @@
       <c r="Z7" s="4" t="n"/>
       <c r="AA7" s="5" t="n"/>
       <c r="AB7" s="4" t="n"/>
-      <c r="AC7" s="4" t="n"/>
+      <c r="AC7" s="5" t="n"/>
       <c r="AD7" s="4" t="n"/>
       <c r="AE7" s="5" t="n"/>
       <c r="AF7" s="4" t="n"/>
@@ -1627,7 +1627,7 @@
       <c r="AZ7" s="5" t="n"/>
       <c r="BA7" s="4" t="n"/>
       <c r="BB7" s="5" t="n"/>
-      <c r="BC7" s="4" t="n"/>
+      <c r="BC7" s="5" t="n"/>
       <c r="BD7" s="5" t="n"/>
       <c r="BE7" s="4" t="n"/>
       <c r="BF7" s="5" t="n"/>
@@ -1654,11 +1654,11 @@
       <c r="CA7" s="5" t="n"/>
       <c r="CB7" s="5" t="n"/>
       <c r="CC7" s="4" t="n"/>
-      <c r="CD7" s="3" t="n"/>
+      <c r="CD7" s="5" t="n"/>
       <c r="CE7" s="4" t="n"/>
       <c r="CF7" s="5" t="n"/>
       <c r="CG7" s="5" t="n"/>
-      <c r="CH7" s="4" t="n"/>
+      <c r="CH7" s="5" t="n"/>
       <c r="CI7" s="4" t="n"/>
       <c r="CJ7" s="4" t="n"/>
       <c r="CK7" s="4" t="n"/>
@@ -1695,12 +1695,12 @@
       <c r="F8" s="5" t="n"/>
       <c r="G8" s="4" t="n"/>
       <c r="H8" s="5" t="n"/>
-      <c r="I8" s="4" t="n"/>
+      <c r="I8" s="5" t="n"/>
       <c r="J8" s="4" t="n"/>
       <c r="K8" s="4" t="n"/>
-      <c r="L8" s="4" t="n"/>
+      <c r="L8" s="5" t="n"/>
       <c r="M8" s="4" t="n"/>
-      <c r="N8" s="4" t="n"/>
+      <c r="N8" s="5" t="n"/>
       <c r="O8" s="5" t="n"/>
       <c r="P8" s="4" t="n"/>
       <c r="Q8" s="4" t="n"/>
@@ -1715,7 +1715,7 @@
       <c r="Z8" s="4" t="n"/>
       <c r="AA8" s="5" t="n"/>
       <c r="AB8" s="4" t="n"/>
-      <c r="AC8" s="4" t="n"/>
+      <c r="AC8" s="5" t="n"/>
       <c r="AD8" s="4" t="n"/>
       <c r="AE8" s="5" t="n"/>
       <c r="AF8" s="4" t="n"/>
@@ -1741,7 +1741,7 @@
       <c r="AZ8" s="5" t="n"/>
       <c r="BA8" s="4" t="n"/>
       <c r="BB8" s="5" t="n"/>
-      <c r="BC8" s="4" t="n"/>
+      <c r="BC8" s="5" t="n"/>
       <c r="BD8" s="5" t="n"/>
       <c r="BE8" s="3" t="n"/>
       <c r="BF8" s="5" t="n"/>
@@ -1772,7 +1772,7 @@
       <c r="CE8" s="3" t="n"/>
       <c r="CF8" s="5" t="n"/>
       <c r="CG8" s="5" t="n"/>
-      <c r="CH8" s="4" t="n"/>
+      <c r="CH8" s="5" t="n"/>
       <c r="CI8" s="4" t="n"/>
       <c r="CJ8" s="4" t="n"/>
       <c r="CK8" s="4" t="n"/>
@@ -1809,12 +1809,12 @@
       <c r="F9" s="5" t="n"/>
       <c r="G9" s="4" t="n"/>
       <c r="H9" s="5" t="n"/>
-      <c r="I9" s="4" t="n"/>
+      <c r="I9" s="5" t="n"/>
       <c r="J9" s="4" t="n"/>
       <c r="K9" s="4" t="n"/>
-      <c r="L9" s="4" t="n"/>
+      <c r="L9" s="5" t="n"/>
       <c r="M9" s="4" t="n"/>
-      <c r="N9" s="4" t="n"/>
+      <c r="N9" s="5" t="n"/>
       <c r="O9" s="5" t="n"/>
       <c r="P9" s="4" t="n"/>
       <c r="Q9" s="4" t="n"/>
@@ -1829,7 +1829,7 @@
       <c r="Z9" s="4" t="n"/>
       <c r="AA9" s="5" t="n"/>
       <c r="AB9" s="4" t="n"/>
-      <c r="AC9" s="4" t="n"/>
+      <c r="AC9" s="5" t="n"/>
       <c r="AD9" s="4" t="n"/>
       <c r="AE9" s="5" t="n"/>
       <c r="AF9" s="4" t="n"/>
@@ -1855,7 +1855,7 @@
       <c r="AZ9" s="5" t="n"/>
       <c r="BA9" s="4" t="n"/>
       <c r="BB9" s="5" t="n"/>
-      <c r="BC9" s="3" t="n"/>
+      <c r="BC9" s="5" t="n"/>
       <c r="BD9" s="5" t="n"/>
       <c r="BE9" s="5" t="n"/>
       <c r="BF9" s="5" t="n"/>
@@ -1886,7 +1886,7 @@
       <c r="CE9" s="5" t="n"/>
       <c r="CF9" s="5" t="n"/>
       <c r="CG9" s="5" t="n"/>
-      <c r="CH9" s="4" t="n"/>
+      <c r="CH9" s="5" t="n"/>
       <c r="CI9" s="4" t="n"/>
       <c r="CJ9" s="4" t="n"/>
       <c r="CK9" s="4" t="n"/>
@@ -1923,12 +1923,12 @@
       <c r="F10" s="5" t="n"/>
       <c r="G10" s="4" t="n"/>
       <c r="H10" s="5" t="n"/>
-      <c r="I10" s="4" t="n"/>
+      <c r="I10" s="5" t="n"/>
       <c r="J10" s="4" t="n"/>
       <c r="K10" s="4" t="n"/>
-      <c r="L10" s="4" t="n"/>
+      <c r="L10" s="5" t="n"/>
       <c r="M10" s="4" t="n"/>
-      <c r="N10" s="4" t="n"/>
+      <c r="N10" s="5" t="n"/>
       <c r="O10" s="5" t="n"/>
       <c r="P10" s="4" t="n"/>
       <c r="Q10" s="4" t="n"/>
@@ -1943,7 +1943,7 @@
       <c r="Z10" s="4" t="n"/>
       <c r="AA10" s="5" t="n"/>
       <c r="AB10" s="4" t="n"/>
-      <c r="AC10" s="4" t="n"/>
+      <c r="AC10" s="5" t="n"/>
       <c r="AD10" s="4" t="n"/>
       <c r="AE10" s="5" t="n"/>
       <c r="AF10" s="4" t="n"/>
@@ -2000,7 +2000,7 @@
       <c r="CE10" s="5" t="n"/>
       <c r="CF10" s="5" t="n"/>
       <c r="CG10" s="5" t="n"/>
-      <c r="CH10" s="4" t="n"/>
+      <c r="CH10" s="5" t="n"/>
       <c r="CI10" s="4" t="n"/>
       <c r="CJ10" s="4" t="n"/>
       <c r="CK10" s="4" t="n"/>
@@ -2037,12 +2037,12 @@
       <c r="F11" s="5" t="n"/>
       <c r="G11" s="4" t="n"/>
       <c r="H11" s="5" t="n"/>
-      <c r="I11" s="4" t="n"/>
+      <c r="I11" s="5" t="n"/>
       <c r="J11" s="4" t="n"/>
       <c r="K11" s="4" t="n"/>
-      <c r="L11" s="4" t="n"/>
+      <c r="L11" s="5" t="n"/>
       <c r="M11" s="4" t="n"/>
-      <c r="N11" s="4" t="n"/>
+      <c r="N11" s="5" t="n"/>
       <c r="O11" s="5" t="n"/>
       <c r="P11" s="4" t="n"/>
       <c r="Q11" s="4" t="n"/>
@@ -2057,7 +2057,7 @@
       <c r="Z11" s="4" t="n"/>
       <c r="AA11" s="5" t="n"/>
       <c r="AB11" s="4" t="n"/>
-      <c r="AC11" s="4" t="n"/>
+      <c r="AC11" s="5" t="n"/>
       <c r="AD11" s="4" t="n"/>
       <c r="AE11" s="5" t="n"/>
       <c r="AF11" s="4" t="n"/>
@@ -2114,7 +2114,7 @@
       <c r="CE11" s="5" t="n"/>
       <c r="CF11" s="5" t="n"/>
       <c r="CG11" s="5" t="n"/>
-      <c r="CH11" s="4" t="n"/>
+      <c r="CH11" s="5" t="n"/>
       <c r="CI11" s="4" t="n"/>
       <c r="CJ11" s="4" t="n"/>
       <c r="CK11" s="4" t="n"/>
@@ -2151,12 +2151,12 @@
       <c r="F12" s="5" t="n"/>
       <c r="G12" s="4" t="n"/>
       <c r="H12" s="5" t="n"/>
-      <c r="I12" s="3" t="n"/>
+      <c r="I12" s="5" t="n"/>
       <c r="J12" s="4" t="n"/>
       <c r="K12" s="4" t="n"/>
-      <c r="L12" s="3" t="n"/>
+      <c r="L12" s="5" t="n"/>
       <c r="M12" s="4" t="n"/>
-      <c r="N12" s="4" t="n"/>
+      <c r="N12" s="5" t="n"/>
       <c r="O12" s="5" t="n"/>
       <c r="P12" s="4" t="n"/>
       <c r="Q12" s="4" t="n"/>
@@ -2171,7 +2171,7 @@
       <c r="Z12" s="4" t="n"/>
       <c r="AA12" s="5" t="n"/>
       <c r="AB12" s="4" t="n"/>
-      <c r="AC12" s="4" t="n"/>
+      <c r="AC12" s="5" t="n"/>
       <c r="AD12" s="4" t="n"/>
       <c r="AE12" s="5" t="n"/>
       <c r="AF12" s="4" t="n"/>
@@ -2228,7 +2228,7 @@
       <c r="CE12" s="5" t="n"/>
       <c r="CF12" s="5" t="n"/>
       <c r="CG12" s="5" t="n"/>
-      <c r="CH12" s="4" t="n"/>
+      <c r="CH12" s="5" t="n"/>
       <c r="CI12" s="4" t="n"/>
       <c r="CJ12" s="4" t="n"/>
       <c r="CK12" s="4" t="n"/>
@@ -2270,7 +2270,7 @@
       <c r="K13" s="4" t="n"/>
       <c r="L13" s="5" t="n"/>
       <c r="M13" s="4" t="n"/>
-      <c r="N13" s="4" t="n"/>
+      <c r="N13" s="5" t="n"/>
       <c r="O13" s="5" t="n"/>
       <c r="P13" s="4" t="n"/>
       <c r="Q13" s="4" t="n"/>
@@ -2285,7 +2285,7 @@
       <c r="Z13" s="4" t="n"/>
       <c r="AA13" s="5" t="n"/>
       <c r="AB13" s="4" t="n"/>
-      <c r="AC13" s="4" t="n"/>
+      <c r="AC13" s="5" t="n"/>
       <c r="AD13" s="4" t="n"/>
       <c r="AE13" s="5" t="n"/>
       <c r="AF13" s="4" t="n"/>
@@ -2342,7 +2342,7 @@
       <c r="CE13" s="5" t="n"/>
       <c r="CF13" s="5" t="n"/>
       <c r="CG13" s="5" t="n"/>
-      <c r="CH13" s="4" t="n"/>
+      <c r="CH13" s="5" t="n"/>
       <c r="CI13" s="4" t="n"/>
       <c r="CJ13" s="4" t="n"/>
       <c r="CK13" s="4" t="n"/>
@@ -2384,7 +2384,7 @@
       <c r="K14" s="4" t="n"/>
       <c r="L14" s="5" t="n"/>
       <c r="M14" s="4" t="n"/>
-      <c r="N14" s="3" t="n"/>
+      <c r="N14" s="5" t="n"/>
       <c r="O14" s="5" t="n"/>
       <c r="P14" s="4" t="n"/>
       <c r="Q14" s="4" t="n"/>
@@ -2399,7 +2399,7 @@
       <c r="Z14" s="4" t="n"/>
       <c r="AA14" s="5" t="n"/>
       <c r="AB14" s="4" t="n"/>
-      <c r="AC14" s="3" t="n"/>
+      <c r="AC14" s="5" t="n"/>
       <c r="AD14" s="4" t="n"/>
       <c r="AE14" s="5" t="n"/>
       <c r="AF14" s="4" t="n"/>
@@ -2456,7 +2456,7 @@
       <c r="CE14" s="5" t="n"/>
       <c r="CF14" s="5" t="n"/>
       <c r="CG14" s="5" t="n"/>
-      <c r="CH14" s="4" t="n"/>
+      <c r="CH14" s="5" t="n"/>
       <c r="CI14" s="4" t="n"/>
       <c r="CJ14" s="4" t="n"/>
       <c r="CK14" s="4" t="n"/>
@@ -2570,7 +2570,7 @@
       <c r="CE15" s="5" t="n"/>
       <c r="CF15" s="5" t="n"/>
       <c r="CG15" s="5" t="n"/>
-      <c r="CH15" s="4" t="n"/>
+      <c r="CH15" s="5" t="n"/>
       <c r="CI15" s="4" t="n"/>
       <c r="CJ15" s="4" t="n"/>
       <c r="CK15" s="4" t="n"/>
@@ -2684,7 +2684,7 @@
       <c r="CE16" s="5" t="n"/>
       <c r="CF16" s="5" t="n"/>
       <c r="CG16" s="5" t="n"/>
-      <c r="CH16" s="3" t="n"/>
+      <c r="CH16" s="5" t="n"/>
       <c r="CI16" s="4" t="n"/>
       <c r="CJ16" s="4" t="n"/>
       <c r="CK16" s="4" t="n"/>

</xml_diff>

<commit_message>
chore: 🗃️ Regenera artefatos apos a mudanca dos arquivos medidos
A matriz de nos muda de verdade, e nao so de data: com o driver de benchmark
fora dos fontes, nos como Add, Assign e Attribute deixam de aparecer em todo
arquivo (vinham do boilerplate, nao das funcoes), entao a cobertura passa a
refletir o que as funcoes de fato exercitam -- 26 das 106 linhas da matriz
mudaram.

Os CSVs trazem os tempos remedidos pelo runner novo; os dois xlsx acompanham
a matriz e o CSV.
</commit_message>
<xml_diff>
--- a/arquivos/xlsx/nos_ast_cobertos.xlsx
+++ b/arquivos/xlsx/nos_ast_cobertos.xlsx
@@ -1011,12 +1011,12 @@
       <c r="F2" s="3" t="n"/>
       <c r="G2" s="4" t="n"/>
       <c r="H2" s="3" t="n"/>
-      <c r="I2" s="3" t="n"/>
+      <c r="I2" s="4" t="n"/>
       <c r="J2" s="4" t="n"/>
       <c r="K2" s="4" t="n"/>
       <c r="L2" s="3" t="n"/>
       <c r="M2" s="4" t="n"/>
-      <c r="N2" s="3" t="n"/>
+      <c r="N2" s="4" t="n"/>
       <c r="O2" s="3" t="n"/>
       <c r="P2" s="4" t="n"/>
       <c r="Q2" s="4" t="n"/>
@@ -1031,13 +1031,13 @@
       <c r="Z2" s="4" t="n"/>
       <c r="AA2" s="3" t="n"/>
       <c r="AB2" s="4" t="n"/>
-      <c r="AC2" s="3" t="n"/>
+      <c r="AC2" s="4" t="n"/>
       <c r="AD2" s="4" t="n"/>
       <c r="AE2" s="4" t="n"/>
       <c r="AF2" s="4" t="n"/>
       <c r="AG2" s="3" t="n"/>
       <c r="AH2" s="4" t="n"/>
-      <c r="AI2" s="3" t="n"/>
+      <c r="AI2" s="4" t="n"/>
       <c r="AJ2" s="4" t="n"/>
       <c r="AK2" s="4" t="n"/>
       <c r="AL2" s="4" t="n"/>
@@ -1054,7 +1054,7 @@
       <c r="AW2" s="3" t="n"/>
       <c r="AX2" s="3" t="n"/>
       <c r="AY2" s="3" t="n"/>
-      <c r="AZ2" s="3" t="n"/>
+      <c r="AZ2" s="4" t="n"/>
       <c r="BA2" s="4" t="n"/>
       <c r="BB2" s="3" t="n"/>
       <c r="BC2" s="3" t="n"/>
@@ -1063,10 +1063,10 @@
       <c r="BF2" s="3" t="n"/>
       <c r="BG2" s="3" t="n"/>
       <c r="BH2" s="4" t="n"/>
-      <c r="BI2" s="3" t="n"/>
+      <c r="BI2" s="4" t="n"/>
       <c r="BJ2" s="3" t="n"/>
       <c r="BK2" s="3" t="n"/>
-      <c r="BL2" s="3" t="n"/>
+      <c r="BL2" s="4" t="n"/>
       <c r="BM2" s="4" t="n"/>
       <c r="BN2" s="4" t="n"/>
       <c r="BO2" s="4" t="n"/>
@@ -1084,11 +1084,11 @@
       <c r="CA2" s="4" t="n"/>
       <c r="CB2" s="3" t="n"/>
       <c r="CC2" s="4" t="n"/>
-      <c r="CD2" s="3" t="n"/>
+      <c r="CD2" s="4" t="n"/>
       <c r="CE2" s="4" t="n"/>
       <c r="CF2" s="4" t="n"/>
-      <c r="CG2" s="3" t="n"/>
-      <c r="CH2" s="3" t="n"/>
+      <c r="CG2" s="4" t="n"/>
+      <c r="CH2" s="4" t="n"/>
       <c r="CI2" s="4" t="n"/>
       <c r="CJ2" s="4" t="n"/>
       <c r="CK2" s="4" t="n"/>
@@ -1105,7 +1105,7 @@
       <c r="CV2" s="4" t="n"/>
       <c r="CW2" s="3" t="n"/>
       <c r="CX2" s="3" t="n"/>
-      <c r="CY2" s="3" t="n"/>
+      <c r="CY2" s="4" t="n"/>
       <c r="CZ2" s="3" t="n"/>
       <c r="DA2" s="4" t="n"/>
       <c r="DB2" s="4" t="n"/>
@@ -1125,12 +1125,12 @@
       <c r="F3" s="5" t="n"/>
       <c r="G3" s="4" t="n"/>
       <c r="H3" s="5" t="n"/>
-      <c r="I3" s="5" t="n"/>
+      <c r="I3" s="4" t="n"/>
       <c r="J3" s="4" t="n"/>
       <c r="K3" s="4" t="n"/>
       <c r="L3" s="5" t="n"/>
       <c r="M3" s="4" t="n"/>
-      <c r="N3" s="5" t="n"/>
+      <c r="N3" s="4" t="n"/>
       <c r="O3" s="5" t="n"/>
       <c r="P3" s="4" t="n"/>
       <c r="Q3" s="4" t="n"/>
@@ -1145,13 +1145,13 @@
       <c r="Z3" s="4" t="n"/>
       <c r="AA3" s="5" t="n"/>
       <c r="AB3" s="4" t="n"/>
-      <c r="AC3" s="5" t="n"/>
+      <c r="AC3" s="4" t="n"/>
       <c r="AD3" s="4" t="n"/>
       <c r="AE3" s="4" t="n"/>
       <c r="AF3" s="4" t="n"/>
       <c r="AG3" s="5" t="n"/>
       <c r="AH3" s="4" t="n"/>
-      <c r="AI3" s="5" t="n"/>
+      <c r="AI3" s="4" t="n"/>
       <c r="AJ3" s="4" t="n"/>
       <c r="AK3" s="4" t="n"/>
       <c r="AL3" s="4" t="n"/>
@@ -1168,7 +1168,7 @@
       <c r="AW3" s="5" t="n"/>
       <c r="AX3" s="5" t="n"/>
       <c r="AY3" s="5" t="n"/>
-      <c r="AZ3" s="5" t="n"/>
+      <c r="AZ3" s="4" t="n"/>
       <c r="BA3" s="4" t="n"/>
       <c r="BB3" s="5" t="n"/>
       <c r="BC3" s="5" t="n"/>
@@ -1177,10 +1177,10 @@
       <c r="BF3" s="5" t="n"/>
       <c r="BG3" s="5" t="n"/>
       <c r="BH3" s="4" t="n"/>
-      <c r="BI3" s="5" t="n"/>
+      <c r="BI3" s="3" t="n"/>
       <c r="BJ3" s="5" t="n"/>
       <c r="BK3" s="5" t="n"/>
-      <c r="BL3" s="5" t="n"/>
+      <c r="BL3" s="4" t="n"/>
       <c r="BM3" s="4" t="n"/>
       <c r="BN3" s="4" t="n"/>
       <c r="BO3" s="4" t="n"/>
@@ -1198,11 +1198,11 @@
       <c r="CA3" s="4" t="n"/>
       <c r="CB3" s="5" t="n"/>
       <c r="CC3" s="4" t="n"/>
-      <c r="CD3" s="5" t="n"/>
+      <c r="CD3" s="4" t="n"/>
       <c r="CE3" s="4" t="n"/>
       <c r="CF3" s="4" t="n"/>
-      <c r="CG3" s="5" t="n"/>
-      <c r="CH3" s="5" t="n"/>
+      <c r="CG3" s="4" t="n"/>
+      <c r="CH3" s="4" t="n"/>
       <c r="CI3" s="4" t="n"/>
       <c r="CJ3" s="4" t="n"/>
       <c r="CK3" s="4" t="n"/>
@@ -1219,7 +1219,7 @@
       <c r="CV3" s="4" t="n"/>
       <c r="CW3" s="5" t="n"/>
       <c r="CX3" s="5" t="n"/>
-      <c r="CY3" s="5" t="n"/>
+      <c r="CY3" s="4" t="n"/>
       <c r="CZ3" s="5" t="n"/>
       <c r="DA3" s="4" t="n"/>
       <c r="DB3" s="4" t="n"/>
@@ -1239,12 +1239,12 @@
       <c r="F4" s="5" t="n"/>
       <c r="G4" s="4" t="n"/>
       <c r="H4" s="5" t="n"/>
-      <c r="I4" s="5" t="n"/>
+      <c r="I4" s="4" t="n"/>
       <c r="J4" s="4" t="n"/>
       <c r="K4" s="4" t="n"/>
       <c r="L4" s="5" t="n"/>
       <c r="M4" s="4" t="n"/>
-      <c r="N4" s="5" t="n"/>
+      <c r="N4" s="4" t="n"/>
       <c r="O4" s="5" t="n"/>
       <c r="P4" s="4" t="n"/>
       <c r="Q4" s="4" t="n"/>
@@ -1259,13 +1259,13 @@
       <c r="Z4" s="4" t="n"/>
       <c r="AA4" s="5" t="n"/>
       <c r="AB4" s="4" t="n"/>
-      <c r="AC4" s="5" t="n"/>
+      <c r="AC4" s="4" t="n"/>
       <c r="AD4" s="4" t="n"/>
       <c r="AE4" s="4" t="n"/>
       <c r="AF4" s="4" t="n"/>
       <c r="AG4" s="5" t="n"/>
       <c r="AH4" s="4" t="n"/>
-      <c r="AI4" s="5" t="n"/>
+      <c r="AI4" s="4" t="n"/>
       <c r="AJ4" s="4" t="n"/>
       <c r="AK4" s="4" t="n"/>
       <c r="AL4" s="4" t="n"/>
@@ -1282,7 +1282,7 @@
       <c r="AW4" s="5" t="n"/>
       <c r="AX4" s="5" t="n"/>
       <c r="AY4" s="5" t="n"/>
-      <c r="AZ4" s="5" t="n"/>
+      <c r="AZ4" s="3" t="n"/>
       <c r="BA4" s="4" t="n"/>
       <c r="BB4" s="5" t="n"/>
       <c r="BC4" s="5" t="n"/>
@@ -1294,7 +1294,7 @@
       <c r="BI4" s="5" t="n"/>
       <c r="BJ4" s="5" t="n"/>
       <c r="BK4" s="5" t="n"/>
-      <c r="BL4" s="5" t="n"/>
+      <c r="BL4" s="4" t="n"/>
       <c r="BM4" s="4" t="n"/>
       <c r="BN4" s="4" t="n"/>
       <c r="BO4" s="4" t="n"/>
@@ -1312,11 +1312,11 @@
       <c r="CA4" s="4" t="n"/>
       <c r="CB4" s="5" t="n"/>
       <c r="CC4" s="4" t="n"/>
-      <c r="CD4" s="5" t="n"/>
+      <c r="CD4" s="4" t="n"/>
       <c r="CE4" s="4" t="n"/>
       <c r="CF4" s="4" t="n"/>
-      <c r="CG4" s="5" t="n"/>
-      <c r="CH4" s="5" t="n"/>
+      <c r="CG4" s="4" t="n"/>
+      <c r="CH4" s="4" t="n"/>
       <c r="CI4" s="4" t="n"/>
       <c r="CJ4" s="4" t="n"/>
       <c r="CK4" s="4" t="n"/>
@@ -1333,7 +1333,7 @@
       <c r="CV4" s="4" t="n"/>
       <c r="CW4" s="5" t="n"/>
       <c r="CX4" s="5" t="n"/>
-      <c r="CY4" s="5" t="n"/>
+      <c r="CY4" s="4" t="n"/>
       <c r="CZ4" s="5" t="n"/>
       <c r="DA4" s="4" t="n"/>
       <c r="DB4" s="3" t="n"/>
@@ -1353,12 +1353,12 @@
       <c r="F5" s="5" t="n"/>
       <c r="G5" s="4" t="n"/>
       <c r="H5" s="5" t="n"/>
-      <c r="I5" s="5" t="n"/>
+      <c r="I5" s="4" t="n"/>
       <c r="J5" s="4" t="n"/>
       <c r="K5" s="4" t="n"/>
       <c r="L5" s="5" t="n"/>
       <c r="M5" s="4" t="n"/>
-      <c r="N5" s="5" t="n"/>
+      <c r="N5" s="4" t="n"/>
       <c r="O5" s="5" t="n"/>
       <c r="P5" s="4" t="n"/>
       <c r="Q5" s="4" t="n"/>
@@ -1373,13 +1373,13 @@
       <c r="Z5" s="4" t="n"/>
       <c r="AA5" s="5" t="n"/>
       <c r="AB5" s="4" t="n"/>
-      <c r="AC5" s="5" t="n"/>
+      <c r="AC5" s="4" t="n"/>
       <c r="AD5" s="4" t="n"/>
       <c r="AE5" s="4" t="n"/>
       <c r="AF5" s="4" t="n"/>
       <c r="AG5" s="5" t="n"/>
       <c r="AH5" s="4" t="n"/>
-      <c r="AI5" s="5" t="n"/>
+      <c r="AI5" s="4" t="n"/>
       <c r="AJ5" s="4" t="n"/>
       <c r="AK5" s="4" t="n"/>
       <c r="AL5" s="4" t="n"/>
@@ -1408,7 +1408,7 @@
       <c r="BI5" s="5" t="n"/>
       <c r="BJ5" s="5" t="n"/>
       <c r="BK5" s="5" t="n"/>
-      <c r="BL5" s="5" t="n"/>
+      <c r="BL5" s="4" t="n"/>
       <c r="BM5" s="3" t="n"/>
       <c r="BN5" s="4" t="n"/>
       <c r="BO5" s="4" t="n"/>
@@ -1426,11 +1426,11 @@
       <c r="CA5" s="4" t="n"/>
       <c r="CB5" s="5" t="n"/>
       <c r="CC5" s="4" t="n"/>
-      <c r="CD5" s="5" t="n"/>
+      <c r="CD5" s="4" t="n"/>
       <c r="CE5" s="4" t="n"/>
       <c r="CF5" s="4" t="n"/>
-      <c r="CG5" s="5" t="n"/>
-      <c r="CH5" s="5" t="n"/>
+      <c r="CG5" s="4" t="n"/>
+      <c r="CH5" s="4" t="n"/>
       <c r="CI5" s="4" t="n"/>
       <c r="CJ5" s="4" t="n"/>
       <c r="CK5" s="4" t="n"/>
@@ -1447,7 +1447,7 @@
       <c r="CV5" s="4" t="n"/>
       <c r="CW5" s="5" t="n"/>
       <c r="CX5" s="5" t="n"/>
-      <c r="CY5" s="5" t="n"/>
+      <c r="CY5" s="4" t="n"/>
       <c r="CZ5" s="5" t="n"/>
       <c r="DA5" s="4" t="n"/>
       <c r="DB5" s="5" t="n"/>
@@ -1467,12 +1467,12 @@
       <c r="F6" s="5" t="n"/>
       <c r="G6" s="4" t="n"/>
       <c r="H6" s="5" t="n"/>
-      <c r="I6" s="5" t="n"/>
+      <c r="I6" s="4" t="n"/>
       <c r="J6" s="4" t="n"/>
       <c r="K6" s="4" t="n"/>
       <c r="L6" s="5" t="n"/>
       <c r="M6" s="4" t="n"/>
-      <c r="N6" s="5" t="n"/>
+      <c r="N6" s="4" t="n"/>
       <c r="O6" s="5" t="n"/>
       <c r="P6" s="4" t="n"/>
       <c r="Q6" s="4" t="n"/>
@@ -1487,13 +1487,13 @@
       <c r="Z6" s="4" t="n"/>
       <c r="AA6" s="5" t="n"/>
       <c r="AB6" s="4" t="n"/>
-      <c r="AC6" s="5" t="n"/>
+      <c r="AC6" s="4" t="n"/>
       <c r="AD6" s="4" t="n"/>
       <c r="AE6" s="3" t="n"/>
       <c r="AF6" s="4" t="n"/>
       <c r="AG6" s="5" t="n"/>
       <c r="AH6" s="4" t="n"/>
-      <c r="AI6" s="5" t="n"/>
+      <c r="AI6" s="4" t="n"/>
       <c r="AJ6" s="4" t="n"/>
       <c r="AK6" s="4" t="n"/>
       <c r="AL6" s="4" t="n"/>
@@ -1522,7 +1522,7 @@
       <c r="BI6" s="5" t="n"/>
       <c r="BJ6" s="5" t="n"/>
       <c r="BK6" s="5" t="n"/>
-      <c r="BL6" s="5" t="n"/>
+      <c r="BL6" s="4" t="n"/>
       <c r="BM6" s="5" t="n"/>
       <c r="BN6" s="4" t="n"/>
       <c r="BO6" s="3" t="n"/>
@@ -1540,11 +1540,11 @@
       <c r="CA6" s="3" t="n"/>
       <c r="CB6" s="5" t="n"/>
       <c r="CC6" s="4" t="n"/>
-      <c r="CD6" s="5" t="n"/>
+      <c r="CD6" s="4" t="n"/>
       <c r="CE6" s="4" t="n"/>
       <c r="CF6" s="3" t="n"/>
-      <c r="CG6" s="5" t="n"/>
-      <c r="CH6" s="5" t="n"/>
+      <c r="CG6" s="3" t="n"/>
+      <c r="CH6" s="4" t="n"/>
       <c r="CI6" s="4" t="n"/>
       <c r="CJ6" s="4" t="n"/>
       <c r="CK6" s="4" t="n"/>
@@ -1561,7 +1561,7 @@
       <c r="CV6" s="4" t="n"/>
       <c r="CW6" s="5" t="n"/>
       <c r="CX6" s="5" t="n"/>
-      <c r="CY6" s="5" t="n"/>
+      <c r="CY6" s="4" t="n"/>
       <c r="CZ6" s="5" t="n"/>
       <c r="DA6" s="4" t="n"/>
       <c r="DB6" s="5" t="n"/>
@@ -1581,12 +1581,12 @@
       <c r="F7" s="5" t="n"/>
       <c r="G7" s="4" t="n"/>
       <c r="H7" s="5" t="n"/>
-      <c r="I7" s="5" t="n"/>
+      <c r="I7" s="4" t="n"/>
       <c r="J7" s="4" t="n"/>
       <c r="K7" s="4" t="n"/>
       <c r="L7" s="5" t="n"/>
       <c r="M7" s="4" t="n"/>
-      <c r="N7" s="5" t="n"/>
+      <c r="N7" s="4" t="n"/>
       <c r="O7" s="5" t="n"/>
       <c r="P7" s="4" t="n"/>
       <c r="Q7" s="4" t="n"/>
@@ -1601,13 +1601,13 @@
       <c r="Z7" s="4" t="n"/>
       <c r="AA7" s="5" t="n"/>
       <c r="AB7" s="4" t="n"/>
-      <c r="AC7" s="5" t="n"/>
+      <c r="AC7" s="4" t="n"/>
       <c r="AD7" s="4" t="n"/>
       <c r="AE7" s="5" t="n"/>
       <c r="AF7" s="4" t="n"/>
       <c r="AG7" s="5" t="n"/>
       <c r="AH7" s="3" t="n"/>
-      <c r="AI7" s="5" t="n"/>
+      <c r="AI7" s="4" t="n"/>
       <c r="AJ7" s="4" t="n"/>
       <c r="AK7" s="4" t="n"/>
       <c r="AL7" s="4" t="n"/>
@@ -1636,7 +1636,7 @@
       <c r="BI7" s="5" t="n"/>
       <c r="BJ7" s="5" t="n"/>
       <c r="BK7" s="5" t="n"/>
-      <c r="BL7" s="5" t="n"/>
+      <c r="BL7" s="4" t="n"/>
       <c r="BM7" s="5" t="n"/>
       <c r="BN7" s="4" t="n"/>
       <c r="BO7" s="5" t="n"/>
@@ -1654,11 +1654,11 @@
       <c r="CA7" s="5" t="n"/>
       <c r="CB7" s="5" t="n"/>
       <c r="CC7" s="4" t="n"/>
-      <c r="CD7" s="5" t="n"/>
+      <c r="CD7" s="3" t="n"/>
       <c r="CE7" s="4" t="n"/>
       <c r="CF7" s="5" t="n"/>
       <c r="CG7" s="5" t="n"/>
-      <c r="CH7" s="5" t="n"/>
+      <c r="CH7" s="4" t="n"/>
       <c r="CI7" s="4" t="n"/>
       <c r="CJ7" s="4" t="n"/>
       <c r="CK7" s="4" t="n"/>
@@ -1675,7 +1675,7 @@
       <c r="CV7" s="4" t="n"/>
       <c r="CW7" s="5" t="n"/>
       <c r="CX7" s="5" t="n"/>
-      <c r="CY7" s="5" t="n"/>
+      <c r="CY7" s="4" t="n"/>
       <c r="CZ7" s="5" t="n"/>
       <c r="DA7" s="4" t="n"/>
       <c r="DB7" s="5" t="n"/>
@@ -1695,12 +1695,12 @@
       <c r="F8" s="5" t="n"/>
       <c r="G8" s="4" t="n"/>
       <c r="H8" s="5" t="n"/>
-      <c r="I8" s="5" t="n"/>
+      <c r="I8" s="4" t="n"/>
       <c r="J8" s="4" t="n"/>
       <c r="K8" s="4" t="n"/>
       <c r="L8" s="5" t="n"/>
       <c r="M8" s="4" t="n"/>
-      <c r="N8" s="5" t="n"/>
+      <c r="N8" s="4" t="n"/>
       <c r="O8" s="5" t="n"/>
       <c r="P8" s="4" t="n"/>
       <c r="Q8" s="4" t="n"/>
@@ -1715,13 +1715,13 @@
       <c r="Z8" s="4" t="n"/>
       <c r="AA8" s="5" t="n"/>
       <c r="AB8" s="4" t="n"/>
-      <c r="AC8" s="5" t="n"/>
+      <c r="AC8" s="4" t="n"/>
       <c r="AD8" s="4" t="n"/>
       <c r="AE8" s="5" t="n"/>
       <c r="AF8" s="4" t="n"/>
       <c r="AG8" s="5" t="n"/>
       <c r="AH8" s="5" t="n"/>
-      <c r="AI8" s="5" t="n"/>
+      <c r="AI8" s="4" t="n"/>
       <c r="AJ8" s="4" t="n"/>
       <c r="AK8" s="4" t="n"/>
       <c r="AL8" s="4" t="n"/>
@@ -1750,7 +1750,7 @@
       <c r="BI8" s="5" t="n"/>
       <c r="BJ8" s="5" t="n"/>
       <c r="BK8" s="5" t="n"/>
-      <c r="BL8" s="5" t="n"/>
+      <c r="BL8" s="4" t="n"/>
       <c r="BM8" s="5" t="n"/>
       <c r="BN8" s="4" t="n"/>
       <c r="BO8" s="5" t="n"/>
@@ -1772,7 +1772,7 @@
       <c r="CE8" s="3" t="n"/>
       <c r="CF8" s="5" t="n"/>
       <c r="CG8" s="5" t="n"/>
-      <c r="CH8" s="5" t="n"/>
+      <c r="CH8" s="4" t="n"/>
       <c r="CI8" s="4" t="n"/>
       <c r="CJ8" s="4" t="n"/>
       <c r="CK8" s="4" t="n"/>
@@ -1789,7 +1789,7 @@
       <c r="CV8" s="4" t="n"/>
       <c r="CW8" s="5" t="n"/>
       <c r="CX8" s="5" t="n"/>
-      <c r="CY8" s="5" t="n"/>
+      <c r="CY8" s="4" t="n"/>
       <c r="CZ8" s="5" t="n"/>
       <c r="DA8" s="4" t="n"/>
       <c r="DB8" s="5" t="n"/>
@@ -1809,12 +1809,12 @@
       <c r="F9" s="5" t="n"/>
       <c r="G9" s="4" t="n"/>
       <c r="H9" s="5" t="n"/>
-      <c r="I9" s="5" t="n"/>
+      <c r="I9" s="4" t="n"/>
       <c r="J9" s="4" t="n"/>
       <c r="K9" s="4" t="n"/>
       <c r="L9" s="5" t="n"/>
       <c r="M9" s="4" t="n"/>
-      <c r="N9" s="5" t="n"/>
+      <c r="N9" s="4" t="n"/>
       <c r="O9" s="5" t="n"/>
       <c r="P9" s="4" t="n"/>
       <c r="Q9" s="4" t="n"/>
@@ -1829,13 +1829,13 @@
       <c r="Z9" s="4" t="n"/>
       <c r="AA9" s="5" t="n"/>
       <c r="AB9" s="4" t="n"/>
-      <c r="AC9" s="5" t="n"/>
+      <c r="AC9" s="4" t="n"/>
       <c r="AD9" s="4" t="n"/>
       <c r="AE9" s="5" t="n"/>
       <c r="AF9" s="4" t="n"/>
       <c r="AG9" s="5" t="n"/>
       <c r="AH9" s="5" t="n"/>
-      <c r="AI9" s="5" t="n"/>
+      <c r="AI9" s="4" t="n"/>
       <c r="AJ9" s="4" t="n"/>
       <c r="AK9" s="4" t="n"/>
       <c r="AL9" s="4" t="n"/>
@@ -1864,7 +1864,7 @@
       <c r="BI9" s="5" t="n"/>
       <c r="BJ9" s="5" t="n"/>
       <c r="BK9" s="5" t="n"/>
-      <c r="BL9" s="5" t="n"/>
+      <c r="BL9" s="4" t="n"/>
       <c r="BM9" s="5" t="n"/>
       <c r="BN9" s="4" t="n"/>
       <c r="BO9" s="5" t="n"/>
@@ -1886,7 +1886,7 @@
       <c r="CE9" s="5" t="n"/>
       <c r="CF9" s="5" t="n"/>
       <c r="CG9" s="5" t="n"/>
-      <c r="CH9" s="5" t="n"/>
+      <c r="CH9" s="4" t="n"/>
       <c r="CI9" s="4" t="n"/>
       <c r="CJ9" s="4" t="n"/>
       <c r="CK9" s="4" t="n"/>
@@ -1903,7 +1903,7 @@
       <c r="CV9" s="4" t="n"/>
       <c r="CW9" s="5" t="n"/>
       <c r="CX9" s="5" t="n"/>
-      <c r="CY9" s="5" t="n"/>
+      <c r="CY9" s="4" t="n"/>
       <c r="CZ9" s="5" t="n"/>
       <c r="DA9" s="4" t="n"/>
       <c r="DB9" s="5" t="n"/>
@@ -1923,12 +1923,12 @@
       <c r="F10" s="5" t="n"/>
       <c r="G10" s="4" t="n"/>
       <c r="H10" s="5" t="n"/>
-      <c r="I10" s="5" t="n"/>
+      <c r="I10" s="4" t="n"/>
       <c r="J10" s="4" t="n"/>
       <c r="K10" s="4" t="n"/>
       <c r="L10" s="5" t="n"/>
       <c r="M10" s="4" t="n"/>
-      <c r="N10" s="5" t="n"/>
+      <c r="N10" s="4" t="n"/>
       <c r="O10" s="5" t="n"/>
       <c r="P10" s="4" t="n"/>
       <c r="Q10" s="4" t="n"/>
@@ -1943,13 +1943,13 @@
       <c r="Z10" s="4" t="n"/>
       <c r="AA10" s="5" t="n"/>
       <c r="AB10" s="4" t="n"/>
-      <c r="AC10" s="5" t="n"/>
+      <c r="AC10" s="4" t="n"/>
       <c r="AD10" s="4" t="n"/>
       <c r="AE10" s="5" t="n"/>
       <c r="AF10" s="4" t="n"/>
       <c r="AG10" s="5" t="n"/>
       <c r="AH10" s="5" t="n"/>
-      <c r="AI10" s="5" t="n"/>
+      <c r="AI10" s="4" t="n"/>
       <c r="AJ10" s="4" t="n"/>
       <c r="AK10" s="4" t="n"/>
       <c r="AL10" s="4" t="n"/>
@@ -1978,7 +1978,7 @@
       <c r="BI10" s="5" t="n"/>
       <c r="BJ10" s="5" t="n"/>
       <c r="BK10" s="5" t="n"/>
-      <c r="BL10" s="5" t="n"/>
+      <c r="BL10" s="4" t="n"/>
       <c r="BM10" s="5" t="n"/>
       <c r="BN10" s="4" t="n"/>
       <c r="BO10" s="5" t="n"/>
@@ -2000,7 +2000,7 @@
       <c r="CE10" s="5" t="n"/>
       <c r="CF10" s="5" t="n"/>
       <c r="CG10" s="5" t="n"/>
-      <c r="CH10" s="5" t="n"/>
+      <c r="CH10" s="4" t="n"/>
       <c r="CI10" s="4" t="n"/>
       <c r="CJ10" s="4" t="n"/>
       <c r="CK10" s="4" t="n"/>
@@ -2017,7 +2017,7 @@
       <c r="CV10" s="4" t="n"/>
       <c r="CW10" s="5" t="n"/>
       <c r="CX10" s="5" t="n"/>
-      <c r="CY10" s="5" t="n"/>
+      <c r="CY10" s="4" t="n"/>
       <c r="CZ10" s="5" t="n"/>
       <c r="DA10" s="4" t="n"/>
       <c r="DB10" s="5" t="n"/>
@@ -2037,12 +2037,12 @@
       <c r="F11" s="5" t="n"/>
       <c r="G11" s="4" t="n"/>
       <c r="H11" s="5" t="n"/>
-      <c r="I11" s="5" t="n"/>
+      <c r="I11" s="4" t="n"/>
       <c r="J11" s="4" t="n"/>
       <c r="K11" s="4" t="n"/>
       <c r="L11" s="5" t="n"/>
       <c r="M11" s="4" t="n"/>
-      <c r="N11" s="5" t="n"/>
+      <c r="N11" s="4" t="n"/>
       <c r="O11" s="5" t="n"/>
       <c r="P11" s="4" t="n"/>
       <c r="Q11" s="4" t="n"/>
@@ -2057,13 +2057,13 @@
       <c r="Z11" s="4" t="n"/>
       <c r="AA11" s="5" t="n"/>
       <c r="AB11" s="4" t="n"/>
-      <c r="AC11" s="5" t="n"/>
+      <c r="AC11" s="4" t="n"/>
       <c r="AD11" s="4" t="n"/>
       <c r="AE11" s="5" t="n"/>
       <c r="AF11" s="4" t="n"/>
       <c r="AG11" s="5" t="n"/>
       <c r="AH11" s="5" t="n"/>
-      <c r="AI11" s="5" t="n"/>
+      <c r="AI11" s="4" t="n"/>
       <c r="AJ11" s="4" t="n"/>
       <c r="AK11" s="4" t="n"/>
       <c r="AL11" s="4" t="n"/>
@@ -2092,7 +2092,7 @@
       <c r="BI11" s="5" t="n"/>
       <c r="BJ11" s="5" t="n"/>
       <c r="BK11" s="5" t="n"/>
-      <c r="BL11" s="5" t="n"/>
+      <c r="BL11" s="4" t="n"/>
       <c r="BM11" s="5" t="n"/>
       <c r="BN11" s="4" t="n"/>
       <c r="BO11" s="5" t="n"/>
@@ -2114,7 +2114,7 @@
       <c r="CE11" s="5" t="n"/>
       <c r="CF11" s="5" t="n"/>
       <c r="CG11" s="5" t="n"/>
-      <c r="CH11" s="5" t="n"/>
+      <c r="CH11" s="4" t="n"/>
       <c r="CI11" s="4" t="n"/>
       <c r="CJ11" s="4" t="n"/>
       <c r="CK11" s="4" t="n"/>
@@ -2131,7 +2131,7 @@
       <c r="CV11" s="4" t="n"/>
       <c r="CW11" s="5" t="n"/>
       <c r="CX11" s="5" t="n"/>
-      <c r="CY11" s="5" t="n"/>
+      <c r="CY11" s="4" t="n"/>
       <c r="CZ11" s="5" t="n"/>
       <c r="DA11" s="4" t="n"/>
       <c r="DB11" s="5" t="n"/>
@@ -2151,12 +2151,12 @@
       <c r="F12" s="5" t="n"/>
       <c r="G12" s="4" t="n"/>
       <c r="H12" s="5" t="n"/>
-      <c r="I12" s="5" t="n"/>
+      <c r="I12" s="3" t="n"/>
       <c r="J12" s="4" t="n"/>
       <c r="K12" s="4" t="n"/>
       <c r="L12" s="5" t="n"/>
       <c r="M12" s="4" t="n"/>
-      <c r="N12" s="5" t="n"/>
+      <c r="N12" s="4" t="n"/>
       <c r="O12" s="5" t="n"/>
       <c r="P12" s="4" t="n"/>
       <c r="Q12" s="4" t="n"/>
@@ -2171,13 +2171,13 @@
       <c r="Z12" s="4" t="n"/>
       <c r="AA12" s="5" t="n"/>
       <c r="AB12" s="4" t="n"/>
-      <c r="AC12" s="5" t="n"/>
+      <c r="AC12" s="4" t="n"/>
       <c r="AD12" s="4" t="n"/>
       <c r="AE12" s="5" t="n"/>
       <c r="AF12" s="4" t="n"/>
       <c r="AG12" s="5" t="n"/>
       <c r="AH12" s="5" t="n"/>
-      <c r="AI12" s="5" t="n"/>
+      <c r="AI12" s="4" t="n"/>
       <c r="AJ12" s="4" t="n"/>
       <c r="AK12" s="4" t="n"/>
       <c r="AL12" s="4" t="n"/>
@@ -2206,7 +2206,7 @@
       <c r="BI12" s="5" t="n"/>
       <c r="BJ12" s="5" t="n"/>
       <c r="BK12" s="5" t="n"/>
-      <c r="BL12" s="5" t="n"/>
+      <c r="BL12" s="4" t="n"/>
       <c r="BM12" s="5" t="n"/>
       <c r="BN12" s="4" t="n"/>
       <c r="BO12" s="5" t="n"/>
@@ -2228,7 +2228,7 @@
       <c r="CE12" s="5" t="n"/>
       <c r="CF12" s="5" t="n"/>
       <c r="CG12" s="5" t="n"/>
-      <c r="CH12" s="5" t="n"/>
+      <c r="CH12" s="4" t="n"/>
       <c r="CI12" s="4" t="n"/>
       <c r="CJ12" s="4" t="n"/>
       <c r="CK12" s="4" t="n"/>
@@ -2245,7 +2245,7 @@
       <c r="CV12" s="4" t="n"/>
       <c r="CW12" s="5" t="n"/>
       <c r="CX12" s="5" t="n"/>
-      <c r="CY12" s="5" t="n"/>
+      <c r="CY12" s="4" t="n"/>
       <c r="CZ12" s="5" t="n"/>
       <c r="DA12" s="4" t="n"/>
       <c r="DB12" s="5" t="n"/>
@@ -2270,7 +2270,7 @@
       <c r="K13" s="4" t="n"/>
       <c r="L13" s="5" t="n"/>
       <c r="M13" s="4" t="n"/>
-      <c r="N13" s="5" t="n"/>
+      <c r="N13" s="4" t="n"/>
       <c r="O13" s="5" t="n"/>
       <c r="P13" s="4" t="n"/>
       <c r="Q13" s="4" t="n"/>
@@ -2285,13 +2285,13 @@
       <c r="Z13" s="4" t="n"/>
       <c r="AA13" s="5" t="n"/>
       <c r="AB13" s="4" t="n"/>
-      <c r="AC13" s="5" t="n"/>
+      <c r="AC13" s="4" t="n"/>
       <c r="AD13" s="4" t="n"/>
       <c r="AE13" s="5" t="n"/>
       <c r="AF13" s="4" t="n"/>
       <c r="AG13" s="5" t="n"/>
       <c r="AH13" s="5" t="n"/>
-      <c r="AI13" s="5" t="n"/>
+      <c r="AI13" s="4" t="n"/>
       <c r="AJ13" s="4" t="n"/>
       <c r="AK13" s="4" t="n"/>
       <c r="AL13" s="4" t="n"/>
@@ -2320,7 +2320,7 @@
       <c r="BI13" s="5" t="n"/>
       <c r="BJ13" s="5" t="n"/>
       <c r="BK13" s="5" t="n"/>
-      <c r="BL13" s="5" t="n"/>
+      <c r="BL13" s="4" t="n"/>
       <c r="BM13" s="5" t="n"/>
       <c r="BN13" s="4" t="n"/>
       <c r="BO13" s="5" t="n"/>
@@ -2342,7 +2342,7 @@
       <c r="CE13" s="5" t="n"/>
       <c r="CF13" s="5" t="n"/>
       <c r="CG13" s="5" t="n"/>
-      <c r="CH13" s="5" t="n"/>
+      <c r="CH13" s="4" t="n"/>
       <c r="CI13" s="4" t="n"/>
       <c r="CJ13" s="4" t="n"/>
       <c r="CK13" s="4" t="n"/>
@@ -2359,7 +2359,7 @@
       <c r="CV13" s="4" t="n"/>
       <c r="CW13" s="5" t="n"/>
       <c r="CX13" s="5" t="n"/>
-      <c r="CY13" s="5" t="n"/>
+      <c r="CY13" s="4" t="n"/>
       <c r="CZ13" s="5" t="n"/>
       <c r="DA13" s="4" t="n"/>
       <c r="DB13" s="5" t="n"/>
@@ -2384,7 +2384,7 @@
       <c r="K14" s="4" t="n"/>
       <c r="L14" s="5" t="n"/>
       <c r="M14" s="4" t="n"/>
-      <c r="N14" s="5" t="n"/>
+      <c r="N14" s="3" t="n"/>
       <c r="O14" s="5" t="n"/>
       <c r="P14" s="4" t="n"/>
       <c r="Q14" s="4" t="n"/>
@@ -2399,13 +2399,13 @@
       <c r="Z14" s="4" t="n"/>
       <c r="AA14" s="5" t="n"/>
       <c r="AB14" s="4" t="n"/>
-      <c r="AC14" s="5" t="n"/>
+      <c r="AC14" s="3" t="n"/>
       <c r="AD14" s="4" t="n"/>
       <c r="AE14" s="5" t="n"/>
       <c r="AF14" s="4" t="n"/>
       <c r="AG14" s="5" t="n"/>
       <c r="AH14" s="5" t="n"/>
-      <c r="AI14" s="5" t="n"/>
+      <c r="AI14" s="4" t="n"/>
       <c r="AJ14" s="4" t="n"/>
       <c r="AK14" s="4" t="n"/>
       <c r="AL14" s="4" t="n"/>
@@ -2434,7 +2434,7 @@
       <c r="BI14" s="5" t="n"/>
       <c r="BJ14" s="5" t="n"/>
       <c r="BK14" s="5" t="n"/>
-      <c r="BL14" s="5" t="n"/>
+      <c r="BL14" s="4" t="n"/>
       <c r="BM14" s="5" t="n"/>
       <c r="BN14" s="3" t="n"/>
       <c r="BO14" s="5" t="n"/>
@@ -2456,7 +2456,7 @@
       <c r="CE14" s="5" t="n"/>
       <c r="CF14" s="5" t="n"/>
       <c r="CG14" s="5" t="n"/>
-      <c r="CH14" s="5" t="n"/>
+      <c r="CH14" s="4" t="n"/>
       <c r="CI14" s="4" t="n"/>
       <c r="CJ14" s="4" t="n"/>
       <c r="CK14" s="4" t="n"/>
@@ -2473,7 +2473,7 @@
       <c r="CV14" s="4" t="n"/>
       <c r="CW14" s="5" t="n"/>
       <c r="CX14" s="5" t="n"/>
-      <c r="CY14" s="5" t="n"/>
+      <c r="CY14" s="4" t="n"/>
       <c r="CZ14" s="5" t="n"/>
       <c r="DA14" s="4" t="n"/>
       <c r="DB14" s="5" t="n"/>
@@ -2519,7 +2519,7 @@
       <c r="AF15" s="4" t="n"/>
       <c r="AG15" s="5" t="n"/>
       <c r="AH15" s="5" t="n"/>
-      <c r="AI15" s="5" t="n"/>
+      <c r="AI15" s="4" t="n"/>
       <c r="AJ15" s="4" t="n"/>
       <c r="AK15" s="4" t="n"/>
       <c r="AL15" s="4" t="n"/>
@@ -2548,7 +2548,7 @@
       <c r="BI15" s="5" t="n"/>
       <c r="BJ15" s="5" t="n"/>
       <c r="BK15" s="5" t="n"/>
-      <c r="BL15" s="5" t="n"/>
+      <c r="BL15" s="4" t="n"/>
       <c r="BM15" s="5" t="n"/>
       <c r="BN15" s="5" t="n"/>
       <c r="BO15" s="5" t="n"/>
@@ -2570,7 +2570,7 @@
       <c r="CE15" s="5" t="n"/>
       <c r="CF15" s="5" t="n"/>
       <c r="CG15" s="5" t="n"/>
-      <c r="CH15" s="5" t="n"/>
+      <c r="CH15" s="4" t="n"/>
       <c r="CI15" s="4" t="n"/>
       <c r="CJ15" s="4" t="n"/>
       <c r="CK15" s="4" t="n"/>
@@ -2587,7 +2587,7 @@
       <c r="CV15" s="4" t="n"/>
       <c r="CW15" s="5" t="n"/>
       <c r="CX15" s="5" t="n"/>
-      <c r="CY15" s="5" t="n"/>
+      <c r="CY15" s="4" t="n"/>
       <c r="CZ15" s="5" t="n"/>
       <c r="DA15" s="4" t="n"/>
       <c r="DB15" s="5" t="n"/>
@@ -2633,7 +2633,7 @@
       <c r="AF16" s="4" t="n"/>
       <c r="AG16" s="5" t="n"/>
       <c r="AH16" s="5" t="n"/>
-      <c r="AI16" s="5" t="n"/>
+      <c r="AI16" s="4" t="n"/>
       <c r="AJ16" s="4" t="n"/>
       <c r="AK16" s="4" t="n"/>
       <c r="AL16" s="4" t="n"/>
@@ -2662,7 +2662,7 @@
       <c r="BI16" s="5" t="n"/>
       <c r="BJ16" s="5" t="n"/>
       <c r="BK16" s="5" t="n"/>
-      <c r="BL16" s="5" t="n"/>
+      <c r="BL16" s="4" t="n"/>
       <c r="BM16" s="5" t="n"/>
       <c r="BN16" s="5" t="n"/>
       <c r="BO16" s="5" t="n"/>
@@ -2684,7 +2684,7 @@
       <c r="CE16" s="5" t="n"/>
       <c r="CF16" s="5" t="n"/>
       <c r="CG16" s="5" t="n"/>
-      <c r="CH16" s="5" t="n"/>
+      <c r="CH16" s="3" t="n"/>
       <c r="CI16" s="4" t="n"/>
       <c r="CJ16" s="4" t="n"/>
       <c r="CK16" s="4" t="n"/>
@@ -2701,7 +2701,7 @@
       <c r="CV16" s="4" t="n"/>
       <c r="CW16" s="5" t="n"/>
       <c r="CX16" s="5" t="n"/>
-      <c r="CY16" s="5" t="n"/>
+      <c r="CY16" s="4" t="n"/>
       <c r="CZ16" s="5" t="n"/>
       <c r="DA16" s="4" t="n"/>
       <c r="DB16" s="5" t="n"/>
@@ -2747,7 +2747,7 @@
       <c r="AF17" s="4" t="n"/>
       <c r="AG17" s="5" t="n"/>
       <c r="AH17" s="5" t="n"/>
-      <c r="AI17" s="5" t="n"/>
+      <c r="AI17" s="4" t="n"/>
       <c r="AJ17" s="4" t="n"/>
       <c r="AK17" s="4" t="n"/>
       <c r="AL17" s="4" t="n"/>
@@ -2776,7 +2776,7 @@
       <c r="BI17" s="5" t="n"/>
       <c r="BJ17" s="5" t="n"/>
       <c r="BK17" s="5" t="n"/>
-      <c r="BL17" s="5" t="n"/>
+      <c r="BL17" s="4" t="n"/>
       <c r="BM17" s="5" t="n"/>
       <c r="BN17" s="5" t="n"/>
       <c r="BO17" s="5" t="n"/>
@@ -2815,7 +2815,7 @@
       <c r="CV17" s="4" t="n"/>
       <c r="CW17" s="5" t="n"/>
       <c r="CX17" s="5" t="n"/>
-      <c r="CY17" s="5" t="n"/>
+      <c r="CY17" s="4" t="n"/>
       <c r="CZ17" s="5" t="n"/>
       <c r="DA17" s="4" t="n"/>
       <c r="DB17" s="5" t="n"/>
@@ -2861,7 +2861,7 @@
       <c r="AF18" s="4" t="n"/>
       <c r="AG18" s="5" t="n"/>
       <c r="AH18" s="5" t="n"/>
-      <c r="AI18" s="5" t="n"/>
+      <c r="AI18" s="4" t="n"/>
       <c r="AJ18" s="4" t="n"/>
       <c r="AK18" s="4" t="n"/>
       <c r="AL18" s="4" t="n"/>
@@ -2890,7 +2890,7 @@
       <c r="BI18" s="5" t="n"/>
       <c r="BJ18" s="5" t="n"/>
       <c r="BK18" s="5" t="n"/>
-      <c r="BL18" s="5" t="n"/>
+      <c r="BL18" s="4" t="n"/>
       <c r="BM18" s="5" t="n"/>
       <c r="BN18" s="5" t="n"/>
       <c r="BO18" s="5" t="n"/>
@@ -2929,7 +2929,7 @@
       <c r="CV18" s="4" t="n"/>
       <c r="CW18" s="5" t="n"/>
       <c r="CX18" s="5" t="n"/>
-      <c r="CY18" s="5" t="n"/>
+      <c r="CY18" s="4" t="n"/>
       <c r="CZ18" s="5" t="n"/>
       <c r="DA18" s="3" t="n"/>
       <c r="DB18" s="5" t="n"/>
@@ -2975,7 +2975,7 @@
       <c r="AF19" s="4" t="n"/>
       <c r="AG19" s="5" t="n"/>
       <c r="AH19" s="5" t="n"/>
-      <c r="AI19" s="5" t="n"/>
+      <c r="AI19" s="4" t="n"/>
       <c r="AJ19" s="4" t="n"/>
       <c r="AK19" s="3" t="n"/>
       <c r="AL19" s="4" t="n"/>
@@ -3004,7 +3004,7 @@
       <c r="BI19" s="5" t="n"/>
       <c r="BJ19" s="5" t="n"/>
       <c r="BK19" s="5" t="n"/>
-      <c r="BL19" s="5" t="n"/>
+      <c r="BL19" s="4" t="n"/>
       <c r="BM19" s="5" t="n"/>
       <c r="BN19" s="5" t="n"/>
       <c r="BO19" s="5" t="n"/>
@@ -3043,7 +3043,7 @@
       <c r="CV19" s="4" t="n"/>
       <c r="CW19" s="5" t="n"/>
       <c r="CX19" s="5" t="n"/>
-      <c r="CY19" s="5" t="n"/>
+      <c r="CY19" s="4" t="n"/>
       <c r="CZ19" s="5" t="n"/>
       <c r="DA19" s="5" t="n"/>
       <c r="DB19" s="5" t="n"/>
@@ -3089,7 +3089,7 @@
       <c r="AF20" s="4" t="n"/>
       <c r="AG20" s="5" t="n"/>
       <c r="AH20" s="5" t="n"/>
-      <c r="AI20" s="5" t="n"/>
+      <c r="AI20" s="4" t="n"/>
       <c r="AJ20" s="4" t="n"/>
       <c r="AK20" s="5" t="n"/>
       <c r="AL20" s="3" t="n"/>
@@ -3118,7 +3118,7 @@
       <c r="BI20" s="5" t="n"/>
       <c r="BJ20" s="5" t="n"/>
       <c r="BK20" s="5" t="n"/>
-      <c r="BL20" s="5" t="n"/>
+      <c r="BL20" s="4" t="n"/>
       <c r="BM20" s="5" t="n"/>
       <c r="BN20" s="5" t="n"/>
       <c r="BO20" s="5" t="n"/>
@@ -3157,7 +3157,7 @@
       <c r="CV20" s="4" t="n"/>
       <c r="CW20" s="5" t="n"/>
       <c r="CX20" s="5" t="n"/>
-      <c r="CY20" s="5" t="n"/>
+      <c r="CY20" s="4" t="n"/>
       <c r="CZ20" s="5" t="n"/>
       <c r="DA20" s="5" t="n"/>
       <c r="DB20" s="5" t="n"/>
@@ -3203,7 +3203,7 @@
       <c r="AF21" s="4" t="n"/>
       <c r="AG21" s="5" t="n"/>
       <c r="AH21" s="5" t="n"/>
-      <c r="AI21" s="5" t="n"/>
+      <c r="AI21" s="4" t="n"/>
       <c r="AJ21" s="4" t="n"/>
       <c r="AK21" s="5" t="n"/>
       <c r="AL21" s="5" t="n"/>
@@ -3232,7 +3232,7 @@
       <c r="BI21" s="5" t="n"/>
       <c r="BJ21" s="5" t="n"/>
       <c r="BK21" s="5" t="n"/>
-      <c r="BL21" s="5" t="n"/>
+      <c r="BL21" s="4" t="n"/>
       <c r="BM21" s="5" t="n"/>
       <c r="BN21" s="5" t="n"/>
       <c r="BO21" s="5" t="n"/>
@@ -3271,7 +3271,7 @@
       <c r="CV21" s="4" t="n"/>
       <c r="CW21" s="5" t="n"/>
       <c r="CX21" s="5" t="n"/>
-      <c r="CY21" s="5" t="n"/>
+      <c r="CY21" s="4" t="n"/>
       <c r="CZ21" s="5" t="n"/>
       <c r="DA21" s="5" t="n"/>
       <c r="DB21" s="5" t="n"/>
@@ -3317,7 +3317,7 @@
       <c r="AF22" s="4" t="n"/>
       <c r="AG22" s="5" t="n"/>
       <c r="AH22" s="5" t="n"/>
-      <c r="AI22" s="5" t="n"/>
+      <c r="AI22" s="4" t="n"/>
       <c r="AJ22" s="4" t="n"/>
       <c r="AK22" s="5" t="n"/>
       <c r="AL22" s="5" t="n"/>
@@ -3346,7 +3346,7 @@
       <c r="BI22" s="5" t="n"/>
       <c r="BJ22" s="5" t="n"/>
       <c r="BK22" s="5" t="n"/>
-      <c r="BL22" s="5" t="n"/>
+      <c r="BL22" s="4" t="n"/>
       <c r="BM22" s="5" t="n"/>
       <c r="BN22" s="5" t="n"/>
       <c r="BO22" s="5" t="n"/>
@@ -3385,7 +3385,7 @@
       <c r="CV22" s="4" t="n"/>
       <c r="CW22" s="5" t="n"/>
       <c r="CX22" s="5" t="n"/>
-      <c r="CY22" s="5" t="n"/>
+      <c r="CY22" s="4" t="n"/>
       <c r="CZ22" s="5" t="n"/>
       <c r="DA22" s="5" t="n"/>
       <c r="DB22" s="5" t="n"/>
@@ -3431,7 +3431,7 @@
       <c r="AF23" s="4" t="n"/>
       <c r="AG23" s="5" t="n"/>
       <c r="AH23" s="5" t="n"/>
-      <c r="AI23" s="5" t="n"/>
+      <c r="AI23" s="4" t="n"/>
       <c r="AJ23" s="4" t="n"/>
       <c r="AK23" s="5" t="n"/>
       <c r="AL23" s="5" t="n"/>
@@ -3460,7 +3460,7 @@
       <c r="BI23" s="5" t="n"/>
       <c r="BJ23" s="5" t="n"/>
       <c r="BK23" s="5" t="n"/>
-      <c r="BL23" s="5" t="n"/>
+      <c r="BL23" s="4" t="n"/>
       <c r="BM23" s="5" t="n"/>
       <c r="BN23" s="5" t="n"/>
       <c r="BO23" s="5" t="n"/>
@@ -3499,7 +3499,7 @@
       <c r="CV23" s="4" t="n"/>
       <c r="CW23" s="5" t="n"/>
       <c r="CX23" s="5" t="n"/>
-      <c r="CY23" s="5" t="n"/>
+      <c r="CY23" s="4" t="n"/>
       <c r="CZ23" s="5" t="n"/>
       <c r="DA23" s="5" t="n"/>
       <c r="DB23" s="5" t="n"/>
@@ -3545,7 +3545,7 @@
       <c r="AF24" s="3" t="n"/>
       <c r="AG24" s="5" t="n"/>
       <c r="AH24" s="5" t="n"/>
-      <c r="AI24" s="5" t="n"/>
+      <c r="AI24" s="3" t="n"/>
       <c r="AJ24" s="4" t="n"/>
       <c r="AK24" s="5" t="n"/>
       <c r="AL24" s="5" t="n"/>
@@ -3574,7 +3574,7 @@
       <c r="BI24" s="5" t="n"/>
       <c r="BJ24" s="5" t="n"/>
       <c r="BK24" s="5" t="n"/>
-      <c r="BL24" s="5" t="n"/>
+      <c r="BL24" s="4" t="n"/>
       <c r="BM24" s="5" t="n"/>
       <c r="BN24" s="5" t="n"/>
       <c r="BO24" s="5" t="n"/>
@@ -3613,7 +3613,7 @@
       <c r="CV24" s="4" t="n"/>
       <c r="CW24" s="5" t="n"/>
       <c r="CX24" s="5" t="n"/>
-      <c r="CY24" s="5" t="n"/>
+      <c r="CY24" s="4" t="n"/>
       <c r="CZ24" s="5" t="n"/>
       <c r="DA24" s="5" t="n"/>
       <c r="DB24" s="5" t="n"/>
@@ -3688,7 +3688,7 @@
       <c r="BI25" s="5" t="n"/>
       <c r="BJ25" s="5" t="n"/>
       <c r="BK25" s="5" t="n"/>
-      <c r="BL25" s="5" t="n"/>
+      <c r="BL25" s="4" t="n"/>
       <c r="BM25" s="5" t="n"/>
       <c r="BN25" s="5" t="n"/>
       <c r="BO25" s="5" t="n"/>
@@ -3727,7 +3727,7 @@
       <c r="CV25" s="4" t="n"/>
       <c r="CW25" s="5" t="n"/>
       <c r="CX25" s="5" t="n"/>
-      <c r="CY25" s="5" t="n"/>
+      <c r="CY25" s="4" t="n"/>
       <c r="CZ25" s="5" t="n"/>
       <c r="DA25" s="5" t="n"/>
       <c r="DB25" s="5" t="n"/>
@@ -3802,7 +3802,7 @@
       <c r="BI26" s="5" t="n"/>
       <c r="BJ26" s="5" t="n"/>
       <c r="BK26" s="5" t="n"/>
-      <c r="BL26" s="5" t="n"/>
+      <c r="BL26" s="4" t="n"/>
       <c r="BM26" s="5" t="n"/>
       <c r="BN26" s="5" t="n"/>
       <c r="BO26" s="5" t="n"/>
@@ -3841,7 +3841,7 @@
       <c r="CV26" s="3" t="n"/>
       <c r="CW26" s="5" t="n"/>
       <c r="CX26" s="5" t="n"/>
-      <c r="CY26" s="5" t="n"/>
+      <c r="CY26" s="4" t="n"/>
       <c r="CZ26" s="5" t="n"/>
       <c r="DA26" s="5" t="n"/>
       <c r="DB26" s="5" t="n"/>
@@ -3916,7 +3916,7 @@
       <c r="BI27" s="5" t="n"/>
       <c r="BJ27" s="5" t="n"/>
       <c r="BK27" s="5" t="n"/>
-      <c r="BL27" s="5" t="n"/>
+      <c r="BL27" s="4" t="n"/>
       <c r="BM27" s="5" t="n"/>
       <c r="BN27" s="5" t="n"/>
       <c r="BO27" s="5" t="n"/>
@@ -3955,7 +3955,7 @@
       <c r="CV27" s="5" t="n"/>
       <c r="CW27" s="5" t="n"/>
       <c r="CX27" s="5" t="n"/>
-      <c r="CY27" s="5" t="n"/>
+      <c r="CY27" s="4" t="n"/>
       <c r="CZ27" s="5" t="n"/>
       <c r="DA27" s="5" t="n"/>
       <c r="DB27" s="5" t="n"/>
@@ -4030,7 +4030,7 @@
       <c r="BI28" s="5" t="n"/>
       <c r="BJ28" s="5" t="n"/>
       <c r="BK28" s="5" t="n"/>
-      <c r="BL28" s="5" t="n"/>
+      <c r="BL28" s="4" t="n"/>
       <c r="BM28" s="5" t="n"/>
       <c r="BN28" s="5" t="n"/>
       <c r="BO28" s="5" t="n"/>
@@ -4069,7 +4069,7 @@
       <c r="CV28" s="5" t="n"/>
       <c r="CW28" s="5" t="n"/>
       <c r="CX28" s="5" t="n"/>
-      <c r="CY28" s="5" t="n"/>
+      <c r="CY28" s="4" t="n"/>
       <c r="CZ28" s="5" t="n"/>
       <c r="DA28" s="5" t="n"/>
       <c r="DB28" s="5" t="n"/>
@@ -4144,7 +4144,7 @@
       <c r="BI29" s="5" t="n"/>
       <c r="BJ29" s="5" t="n"/>
       <c r="BK29" s="5" t="n"/>
-      <c r="BL29" s="5" t="n"/>
+      <c r="BL29" s="3" t="n"/>
       <c r="BM29" s="5" t="n"/>
       <c r="BN29" s="5" t="n"/>
       <c r="BO29" s="5" t="n"/>
@@ -4183,7 +4183,7 @@
       <c r="CV29" s="5" t="n"/>
       <c r="CW29" s="5" t="n"/>
       <c r="CX29" s="5" t="n"/>
-      <c r="CY29" s="5" t="n"/>
+      <c r="CY29" s="3" t="n"/>
       <c r="CZ29" s="5" t="n"/>
       <c r="DA29" s="5" t="n"/>
       <c r="DB29" s="5" t="n"/>

</xml_diff>